<commit_message>
Update GOOGL data - 2026-09-06 05:42:48
</commit_message>
<xml_diff>
--- a/data/GOOGL_data.xlsx
+++ b/data/GOOGL_data.xlsx
@@ -4839,7 +4839,7 @@
         <v>22.785429</v>
       </c>
       <c r="M2" t="n">
-        <v>19.93</v>
+        <v>19.94</v>
       </c>
       <c r="N2" t="n">
         <v>408.61</v>
@@ -4897,7 +4897,7 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>2026-09-06 05:34:41</t>
+          <t>2026-09-06 05:41:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update GOOGL data - 2026-09-06 16:10:47
</commit_message>
<xml_diff>
--- a/data/GOOGL_data.xlsx
+++ b/data/GOOGL_data.xlsx
@@ -4652,7 +4652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AF2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4773,25 +4773,45 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>book_value</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>price_to_book</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>earnings_growth</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>shares_outstanding</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
           <t>sector</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -4875,29 +4895,41 @@
       <c r="W2" t="n">
         <v>2.724</v>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X2" t="n">
+        <v>50.896</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>6.650031</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>5867155790</v>
+      </c>
+      <c r="AB2" t="inlineStr">
         <is>
           <t>Communication Services</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>Internet Content &amp; Information</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>https://abc.xyz</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Alphabet Inc. offers various products and platforms in the United States, Europe, the Middle East, Africa, the Asia-Pacific, Canada, and Latin America. It operates through Google Services, Google Cloud, and Other Bets segments. The Google Services segment provides products and services, including ads, Android, Chrome, devices, Gmail, Google Drive, Google Maps, Google Photos, Google Play, Search, and YouTube. It is also involved in the sale of apps and in-app purchases and digital content in Google Play and YouTube; and devices, as well as the provision of YouTube consumer subscription services, such as YouTube TV, YouTube Music and Premium, NFL Sunday Ticket, and Google One. The Google Cloud segment offers consumption-based fees and subscriptions for AI solutions, including AI infrastructure, Vertex AI platform, and Gemini enterprise. It also provides cybersecurity, and data and analytics services; Google Workspace that include cloud-based communication and collaboration tools for enterprises, such as Calendar, Gmail, Docs, Drive, and Meet; and other enterprise services. The Other Bets segment sells transportation and internet services. Alphabet Inc. was incorporated in 1998 and is headquartered in Mountain View, California.</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>2026-09-06 05:41:42</t>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>2026-09-06 16:09:45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update GOOGL data - 2026-09-06 17:00:22
</commit_message>
<xml_diff>
--- a/data/GOOGL_data.xlsx
+++ b/data/GOOGL_data.xlsx
@@ -4873,15 +4873,11 @@
       <c r="Q2" t="n">
         <v>0.26</v>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="R2" t="n">
+        <v>0.54771</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.34033</v>
       </c>
       <c r="T2" t="n">
         <v>0.48676</v>
@@ -4929,7 +4925,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>2026-09-06 16:48:50</t>
+          <t>2026-09-06 16:59:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update GOOGL data - 2026-09-06 22:21:27
</commit_message>
<xml_diff>
--- a/data/GOOGL_data.xlsx
+++ b/data/GOOGL_data.xlsx
@@ -4652,7 +4652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:AI2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4793,25 +4793,40 @@
       </c>
       <c r="AB1" t="inlineStr">
         <is>
+          <t>total_revenue</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>enterprise_value</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>ebitda</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>sector</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -4903,29 +4918,38 @@
       <c r="AA2" t="n">
         <v>5867155790</v>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AB2" t="n">
+        <v>445865984000</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>4035705831424</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>173164003328</v>
+      </c>
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Communication Services</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>Internet Content &amp; Information</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>https://abc.xyz</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>Alphabet Inc. offers various products and platforms in the United States, Europe, the Middle East, Africa, the Asia-Pacific, Canada, and Latin America. It operates through Google Services, Google Cloud, and Other Bets segments. The Google Services segment provides products and services, including ads, Android, Chrome, devices, Gmail, Google Drive, Google Maps, Google Photos, Google Play, Search, and YouTube. It is also involved in the sale of apps and in-app purchases and digital content in Google Play and YouTube; and devices, as well as the provision of YouTube consumer subscription services, such as YouTube TV, YouTube Music and Premium, NFL Sunday Ticket, and Google One. The Google Cloud segment offers consumption-based fees and subscriptions for AI solutions, including AI infrastructure, Vertex AI platform, and Gemini enterprise. It also provides cybersecurity, and data and analytics services; Google Workspace that include cloud-based communication and collaboration tools for enterprises, such as Calendar, Gmail, Docs, Drive, and Meet; and other enterprise services. The Other Bets segment sells transportation and internet services. Alphabet Inc. was incorporated in 1998 and is headquartered in Mountain View, California.</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>2026-09-06 16:59:20</t>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>2026-09-06 22:20:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update GOOGL data - 2026-09-08 08:53:13
</commit_message>
<xml_diff>
--- a/data/GOOGL_data.xlsx
+++ b/data/GOOGL_data.xlsx
@@ -472,16 +472,16 @@
         <v>45905</v>
       </c>
       <c r="B2" t="n">
-        <v>231.3907550155185</v>
+        <v>231.3907399385365</v>
       </c>
       <c r="C2" t="n">
-        <v>234.9383456001989</v>
+        <v>234.9383302920627</v>
       </c>
       <c r="D2" t="n">
-        <v>231.091797506623</v>
+        <v>231.0917824491205</v>
       </c>
       <c r="E2" t="n">
-        <v>234.1809997558594</v>
+        <v>234.1809844970703</v>
       </c>
       <c r="F2" t="n">
         <v>46588900</v>
@@ -498,16 +498,16 @@
         <v>45908</v>
       </c>
       <c r="B3" t="n">
-        <v>234.8592056813389</v>
+        <v>234.8592210333607</v>
       </c>
       <c r="C3" t="n">
-        <v>237.512309448077</v>
+        <v>237.512324973524</v>
       </c>
       <c r="D3" t="n">
-        <v>233.0638717332001</v>
+        <v>233.0638869678665</v>
       </c>
       <c r="E3" t="n">
-        <v>233.4329071044922</v>
+        <v>233.4329223632812</v>
       </c>
       <c r="F3" t="n">
         <v>32474700</v>
@@ -524,16 +524,16 @@
         <v>45909</v>
       </c>
       <c r="B4" t="n">
-        <v>233.5625640692738</v>
+        <v>233.562578980389</v>
       </c>
       <c r="C4" t="n">
-        <v>239.8462249904786</v>
+        <v>239.8462403027557</v>
       </c>
       <c r="D4" t="n">
-        <v>232.6249999826575</v>
+        <v>232.6250148339166</v>
       </c>
       <c r="E4" t="n">
-        <v>239.0084075927734</v>
+        <v>239.0084228515625</v>
       </c>
       <c r="F4" t="n">
         <v>38061000</v>
@@ -576,16 +576,16 @@
         <v>45911</v>
       </c>
       <c r="B6" t="n">
-        <v>239.2577712479691</v>
+        <v>239.2577864756533</v>
       </c>
       <c r="C6" t="n">
-        <v>241.6216187469878</v>
+        <v>241.6216341251204</v>
       </c>
       <c r="D6" t="n">
-        <v>235.6371823693535</v>
+        <v>235.6371973666035</v>
       </c>
       <c r="E6" t="n">
-        <v>239.7464904785156</v>
+        <v>239.7465057373047</v>
       </c>
       <c r="F6" t="n">
         <v>30599300</v>
@@ -628,16 +628,16 @@
         <v>45915</v>
       </c>
       <c r="B8" t="n">
-        <v>244.0253822711298</v>
+        <v>244.0253674338205</v>
       </c>
       <c r="C8" t="n">
-        <v>251.7552796155814</v>
+        <v>251.7552643082765</v>
       </c>
       <c r="D8" t="n">
-        <v>244.0253822711298</v>
+        <v>244.0253674338205</v>
       </c>
       <c r="E8" t="n">
-        <v>250.9573516845703</v>
+        <v>250.9573364257812</v>
       </c>
       <c r="F8" t="n">
         <v>58383800</v>
@@ -654,16 +654,16 @@
         <v>45916</v>
       </c>
       <c r="B9" t="n">
-        <v>251.4261108558069</v>
+        <v>251.4261261704888</v>
       </c>
       <c r="C9" t="n">
-        <v>252.3836121103763</v>
+        <v>252.3836274833809</v>
       </c>
       <c r="D9" t="n">
-        <v>248.8228805399337</v>
+        <v>248.8228956960496</v>
       </c>
       <c r="E9" t="n">
-        <v>250.5084991455078</v>
+        <v>250.5085144042969</v>
       </c>
       <c r="F9" t="n">
         <v>34109700</v>
@@ -706,16 +706,16 @@
         <v>45918</v>
       </c>
       <c r="B11" t="n">
-        <v>251.0271530076639</v>
+        <v>251.0271682452624</v>
       </c>
       <c r="C11" t="n">
-        <v>253.3311738191467</v>
+        <v>253.3311891966015</v>
       </c>
       <c r="D11" t="n">
-        <v>249.1520399405299</v>
+        <v>249.1520550643071</v>
       </c>
       <c r="E11" t="n">
-        <v>251.3762512207031</v>
+        <v>251.3762664794922</v>
       </c>
       <c r="F11" t="n">
         <v>31239500</v>
@@ -732,16 +732,16 @@
         <v>45919</v>
       </c>
       <c r="B12" t="n">
-        <v>252.5930922260568</v>
+        <v>252.5931073967866</v>
       </c>
       <c r="C12" t="n">
-        <v>255.3359589728353</v>
+        <v>255.3359743083016</v>
       </c>
       <c r="D12" t="n">
-        <v>251.1568250217611</v>
+        <v>251.1568401062288</v>
       </c>
       <c r="E12" t="n">
-        <v>254.0592803955078</v>
+        <v>254.0592956542969</v>
       </c>
       <c r="F12" t="n">
         <v>55571400</v>
@@ -914,16 +914,16 @@
         <v>45930</v>
       </c>
       <c r="B19" t="n">
-        <v>242.1801651040411</v>
+        <v>242.180180344627</v>
       </c>
       <c r="C19" t="n">
-        <v>242.6589157556348</v>
+        <v>242.6589310263489</v>
       </c>
       <c r="D19" t="n">
-        <v>238.6294019345709</v>
+        <v>238.6294169517045</v>
       </c>
       <c r="E19" t="n">
-        <v>242.4694213867188</v>
+        <v>242.4694366455078</v>
       </c>
       <c r="F19" t="n">
         <v>34724300</v>
@@ -966,16 +966,16 @@
         <v>45932</v>
       </c>
       <c r="B21" t="n">
-        <v>244.5140808226371</v>
+        <v>244.5140960478885</v>
       </c>
       <c r="C21" t="n">
-        <v>246.1697784759451</v>
+        <v>246.1697938042925</v>
       </c>
       <c r="D21" t="n">
-        <v>241.6714827842888</v>
+        <v>241.671497832539</v>
       </c>
       <c r="E21" t="n">
-        <v>245.0526885986328</v>
+        <v>245.0527038574219</v>
       </c>
       <c r="F21" t="n">
         <v>25483300</v>
@@ -992,16 +992,16 @@
         <v>45933</v>
       </c>
       <c r="B22" t="n">
-        <v>243.8558378805103</v>
+        <v>243.8558226752064</v>
       </c>
       <c r="C22" t="n">
-        <v>245.6611405975774</v>
+        <v>245.6611252797062</v>
       </c>
       <c r="D22" t="n">
-        <v>241.0331766174326</v>
+        <v>241.0331615881319</v>
       </c>
       <c r="E22" t="n">
-        <v>244.7136077880859</v>
+        <v>244.7135925292969</v>
       </c>
       <c r="F22" t="n">
         <v>30249600</v>
@@ -1044,16 +1044,16 @@
         <v>45937</v>
       </c>
       <c r="B24" t="n">
-        <v>247.6260272338786</v>
+        <v>247.6260118192477</v>
       </c>
       <c r="C24" t="n">
-        <v>249.7903967365714</v>
+        <v>249.7903811872092</v>
       </c>
       <c r="D24" t="n">
-        <v>244.8831603422913</v>
+        <v>244.8831450984028</v>
       </c>
       <c r="E24" t="n">
-        <v>245.1225280761719</v>
+        <v>245.1225128173828</v>
       </c>
       <c r="F24" t="n">
         <v>23181300</v>
@@ -1070,16 +1070,16 @@
         <v>45938</v>
       </c>
       <c r="B25" t="n">
-        <v>244.3245879910796</v>
+        <v>244.3246032710778</v>
       </c>
       <c r="C25" t="n">
-        <v>245.3718521480096</v>
+        <v>245.3718674935034</v>
       </c>
       <c r="D25" t="n">
-        <v>243.1875457247831</v>
+        <v>243.187560933671</v>
       </c>
       <c r="E25" t="n">
-        <v>243.9854583740234</v>
+        <v>243.9854736328125</v>
       </c>
       <c r="F25" t="n">
         <v>21307100</v>
@@ -1148,16 +1148,16 @@
         <v>45943</v>
       </c>
       <c r="B28" t="n">
-        <v>239.5869258671789</v>
+        <v>239.5869408797282</v>
       </c>
       <c r="C28" t="n">
-        <v>243.8657913377574</v>
+        <v>243.865806618421</v>
       </c>
       <c r="D28" t="n">
-        <v>239.0882228174084</v>
+        <v>239.0882377987089</v>
       </c>
       <c r="E28" t="n">
-        <v>243.5166931152344</v>
+        <v>243.5167083740234</v>
       </c>
       <c r="F28" t="n">
         <v>24995000</v>
@@ -1200,16 +1200,16 @@
         <v>45945</v>
       </c>
       <c r="B30" t="n">
-        <v>246.6086514775368</v>
+        <v>246.6086665065597</v>
       </c>
       <c r="C30" t="n">
-        <v>251.4560455996756</v>
+        <v>251.4560609241123</v>
       </c>
       <c r="D30" t="n">
-        <v>245.3519253048375</v>
+        <v>245.3519402572719</v>
       </c>
       <c r="E30" t="n">
-        <v>250.3788452148438</v>
+        <v>250.3788604736328</v>
       </c>
       <c r="F30" t="n">
         <v>27007700</v>
@@ -1252,16 +1252,16 @@
         <v>45947</v>
       </c>
       <c r="B32" t="n">
-        <v>250.1095547697768</v>
+        <v>250.1095396639979</v>
       </c>
       <c r="C32" t="n">
-        <v>253.5605866634714</v>
+        <v>253.5605713492617</v>
       </c>
       <c r="D32" t="n">
-        <v>247.1672097408255</v>
+        <v>247.1671948127543</v>
       </c>
       <c r="E32" t="n">
-        <v>252.6429748535156</v>
+        <v>252.6429595947266</v>
       </c>
       <c r="F32" t="n">
         <v>29671600</v>
@@ -1330,16 +1330,16 @@
         <v>45952</v>
       </c>
       <c r="B35" t="n">
-        <v>253.7101963156115</v>
+        <v>253.710180894347</v>
       </c>
       <c r="C35" t="n">
-        <v>255.6950248045094</v>
+        <v>255.6950092626011</v>
       </c>
       <c r="D35" t="n">
-        <v>248.6433712710665</v>
+        <v>248.6433561577788</v>
       </c>
       <c r="E35" t="n">
-        <v>251.0371551513672</v>
+        <v>251.0371398925781</v>
       </c>
       <c r="F35" t="n">
         <v>35029400</v>
@@ -1382,16 +1382,16 @@
         <v>45954</v>
       </c>
       <c r="B37" t="n">
-        <v>255.9144256499636</v>
+        <v>255.9144859008052</v>
       </c>
       <c r="C37" t="n">
-        <v>261.0012024879728</v>
+        <v>261.0012639364123</v>
       </c>
       <c r="D37" t="n">
-        <v>254.6577147509474</v>
+        <v>254.6577747059171</v>
       </c>
       <c r="E37" t="n">
-        <v>259.2457885742188</v>
+        <v>259.245849609375</v>
       </c>
       <c r="F37" t="n">
         <v>28655100</v>
@@ -1408,16 +1408,16 @@
         <v>45957</v>
       </c>
       <c r="B38" t="n">
-        <v>264.1330942614516</v>
+        <v>264.1330642482098</v>
       </c>
       <c r="C38" t="n">
-        <v>269.4393020900735</v>
+        <v>269.4392714738914</v>
       </c>
       <c r="D38" t="n">
-        <v>263.5944864374467</v>
+        <v>263.5944564854066</v>
       </c>
       <c r="E38" t="n">
-        <v>268.571533203125</v>
+        <v>268.5715026855469</v>
       </c>
       <c r="F38" t="n">
         <v>35235200</v>
@@ -1434,16 +1434,16 @@
         <v>45958</v>
       </c>
       <c r="B39" t="n">
-        <v>268.9904266199372</v>
+        <v>268.9904573908112</v>
       </c>
       <c r="C39" t="n">
-        <v>270.0277373828665</v>
+        <v>270.0277682724026</v>
       </c>
       <c r="D39" t="n">
-        <v>265.8086990443333</v>
+        <v>265.808729451237</v>
       </c>
       <c r="E39" t="n">
-        <v>266.7761840820312</v>
+        <v>266.7762145996094</v>
       </c>
       <c r="F39" t="n">
         <v>29738600</v>
@@ -1460,16 +1460,16 @@
         <v>45959</v>
       </c>
       <c r="B40" t="n">
-        <v>267.055471479175</v>
+        <v>267.0555012387311</v>
       </c>
       <c r="C40" t="n">
-        <v>274.6257797911847</v>
+        <v>274.6258103943446</v>
       </c>
       <c r="D40" t="n">
-        <v>266.975692387603</v>
+        <v>266.9757221382688</v>
       </c>
       <c r="E40" t="n">
-        <v>273.8577880859375</v>
+        <v>273.8578186035156</v>
       </c>
       <c r="F40" t="n">
         <v>43580300</v>
@@ -1486,16 +1486,16 @@
         <v>45960</v>
       </c>
       <c r="B41" t="n">
-        <v>290.8336389163956</v>
+        <v>290.8336705300809</v>
       </c>
       <c r="C41" t="n">
-        <v>290.8336389163956</v>
+        <v>290.8336705300809</v>
       </c>
       <c r="D41" t="n">
-        <v>279.3335478851562</v>
+        <v>279.3335782487789</v>
       </c>
       <c r="E41" t="n">
-        <v>280.7498779296875</v>
+        <v>280.7499084472656</v>
       </c>
       <c r="F41" t="n">
         <v>74876000</v>
@@ -1564,16 +1564,16 @@
         <v>45965</v>
       </c>
       <c r="B44" t="n">
-        <v>276.0321395313242</v>
+        <v>276.032169962035</v>
       </c>
       <c r="C44" t="n">
-        <v>280.5404041676455</v>
+        <v>280.5404350953626</v>
       </c>
       <c r="D44" t="n">
-        <v>275.5434202802167</v>
+        <v>275.5434506570495</v>
       </c>
       <c r="E44" t="n">
-        <v>276.8200988769531</v>
+        <v>276.8201293945312</v>
       </c>
       <c r="F44" t="n">
         <v>30078400</v>
@@ -1616,16 +1616,16 @@
         <v>45967</v>
       </c>
       <c r="B46" t="n">
-        <v>284.5898651937554</v>
+        <v>284.5898957734926</v>
       </c>
       <c r="C46" t="n">
-        <v>287.6020510547858</v>
+        <v>287.6020819581881</v>
       </c>
       <c r="D46" t="n">
-        <v>280.4107616957575</v>
+        <v>280.4107918264418</v>
       </c>
       <c r="E46" t="n">
-        <v>284.0113830566406</v>
+        <v>284.0114135742188</v>
       </c>
       <c r="F46" t="n">
         <v>37173600</v>
@@ -1642,16 +1642,16 @@
         <v>45968</v>
       </c>
       <c r="B47" t="n">
-        <v>282.4753944065927</v>
+        <v>282.4753324126648</v>
       </c>
       <c r="C47" t="n">
-        <v>283.0439232317803</v>
+        <v>283.0438611130793</v>
       </c>
       <c r="D47" t="n">
-        <v>274.4762078378772</v>
+        <v>274.4761475995039</v>
       </c>
       <c r="E47" t="n">
-        <v>278.1067504882812</v>
+        <v>278.106689453125</v>
       </c>
       <c r="F47" t="n">
         <v>34479600</v>
@@ -1720,16 +1720,16 @@
         <v>45973</v>
       </c>
       <c r="B50" t="n">
-        <v>290.9234183741868</v>
+        <v>290.9233873275988</v>
       </c>
       <c r="C50" t="n">
-        <v>291.2525794490294</v>
+        <v>291.2525483673142</v>
       </c>
       <c r="D50" t="n">
-        <v>282.9541529801612</v>
+        <v>282.9541227840324</v>
       </c>
       <c r="E50" t="n">
-        <v>285.96630859375</v>
+        <v>285.9662780761719</v>
       </c>
       <c r="F50" t="n">
         <v>24829900</v>
@@ -1746,16 +1746,16 @@
         <v>45974</v>
       </c>
       <c r="B51" t="n">
-        <v>281.6076529103283</v>
+        <v>281.6076219797447</v>
       </c>
       <c r="C51" t="n">
-        <v>282.1063559927165</v>
+        <v>282.1063250073575</v>
       </c>
       <c r="D51" t="n">
-        <v>276.5208753822851</v>
+        <v>276.5208450104115</v>
       </c>
       <c r="E51" t="n">
-        <v>277.8474426269531</v>
+        <v>277.847412109375</v>
       </c>
       <c r="F51" t="n">
         <v>29494000</v>
@@ -1772,16 +1772,16 @@
         <v>45975</v>
       </c>
       <c r="B52" t="n">
-        <v>270.705963217399</v>
+        <v>270.7059931829425</v>
       </c>
       <c r="C52" t="n">
-        <v>277.8374099534448</v>
+        <v>277.8374407083971</v>
       </c>
       <c r="D52" t="n">
-        <v>269.997813487729</v>
+        <v>269.9978433748846</v>
       </c>
       <c r="E52" t="n">
-        <v>275.6929931640625</v>
+        <v>275.6930236816406</v>
       </c>
       <c r="F52" t="n">
         <v>31647200</v>
@@ -1798,16 +1798,16 @@
         <v>45978</v>
       </c>
       <c r="B53" t="n">
-        <v>285.0387085276487</v>
+        <v>285.038677928695</v>
       </c>
       <c r="C53" t="n">
-        <v>293.1875295999499</v>
+        <v>293.1874981262189</v>
       </c>
       <c r="D53" t="n">
-        <v>282.8344496120375</v>
+        <v>282.8344192497114</v>
       </c>
       <c r="E53" t="n">
-        <v>284.2806701660156</v>
+        <v>284.2806396484375</v>
       </c>
       <c r="F53" t="n">
         <v>52670200</v>
@@ -1902,16 +1902,16 @@
         <v>45982</v>
       </c>
       <c r="B57" t="n">
-        <v>295.6511348655125</v>
+        <v>295.6511046778972</v>
       </c>
       <c r="C57" t="n">
-        <v>303.1316807498811</v>
+        <v>303.1316497984607</v>
       </c>
       <c r="D57" t="n">
-        <v>293.0877938372482</v>
+        <v>293.0877639113642</v>
       </c>
       <c r="E57" t="n">
-        <v>298.8827209472656</v>
+        <v>298.8826904296875</v>
       </c>
       <c r="F57" t="n">
         <v>74137700</v>
@@ -1980,16 +1980,16 @@
         <v>45987</v>
       </c>
       <c r="B60" t="n">
-        <v>319.8481736259059</v>
+        <v>319.8482042131112</v>
       </c>
       <c r="C60" t="n">
-        <v>323.6582721471574</v>
+        <v>323.658303098724</v>
       </c>
       <c r="D60" t="n">
-        <v>315.9682798124272</v>
+        <v>315.9683100285969</v>
       </c>
       <c r="E60" t="n">
-        <v>319.1200866699219</v>
+        <v>319.1201171875</v>
       </c>
       <c r="F60" t="n">
         <v>51373400</v>
@@ -2006,16 +2006,16 @@
         <v>45989</v>
       </c>
       <c r="B61" t="n">
-        <v>322.5311844719001</v>
+        <v>322.5312152935296</v>
       </c>
       <c r="C61" t="n">
-        <v>326.0021684294219</v>
+        <v>326.0021995827445</v>
       </c>
       <c r="D61" t="n">
-        <v>315.9682661584897</v>
+        <v>315.9682963529555</v>
       </c>
       <c r="E61" t="n">
-        <v>319.3494567871094</v>
+        <v>319.3494873046875</v>
       </c>
       <c r="F61" t="n">
         <v>26018600</v>
@@ -2032,16 +2032,16 @@
         <v>45992</v>
       </c>
       <c r="B62" t="n">
-        <v>316.8759510785769</v>
+        <v>316.8759202886677</v>
       </c>
       <c r="C62" t="n">
-        <v>319.020368247556</v>
+        <v>319.02033724928</v>
       </c>
       <c r="D62" t="n">
-        <v>313.0758360216101</v>
+        <v>313.075805600947</v>
       </c>
       <c r="E62" t="n">
-        <v>314.0732421875</v>
+        <v>314.0732116699219</v>
       </c>
       <c r="F62" t="n">
         <v>41183000</v>
@@ -2058,16 +2058,16 @@
         <v>45993</v>
       </c>
       <c r="B63" t="n">
-        <v>315.9184251730286</v>
+        <v>315.9183945655827</v>
       </c>
       <c r="C63" t="n">
-        <v>317.5541859262309</v>
+        <v>317.554155160306</v>
       </c>
       <c r="D63" t="n">
-        <v>313.095779063488</v>
+        <v>313.0957487295115</v>
       </c>
       <c r="E63" t="n">
-        <v>314.9908447265625</v>
+        <v>314.9908142089844</v>
       </c>
       <c r="F63" t="n">
         <v>35854700</v>
@@ -2084,16 +2084,16 @@
         <v>45994</v>
       </c>
       <c r="B64" t="n">
-        <v>315.0706445626379</v>
+        <v>315.0706144021458</v>
       </c>
       <c r="C64" t="n">
-        <v>320.7458575749233</v>
+        <v>320.7458268711651</v>
       </c>
       <c r="D64" t="n">
-        <v>313.2852790244178</v>
+        <v>313.2852490348319</v>
       </c>
       <c r="E64" t="n">
-        <v>318.8009338378906</v>
+        <v>318.8009033203125</v>
       </c>
       <c r="F64" t="n">
         <v>41838300</v>
@@ -2110,16 +2110,16 @@
         <v>45995</v>
       </c>
       <c r="B65" t="n">
-        <v>321.3941698854088</v>
+        <v>321.3942008459266</v>
       </c>
       <c r="C65" t="n">
-        <v>321.5238071066378</v>
+        <v>321.5238380796439</v>
       </c>
       <c r="D65" t="n">
-        <v>313.8837033726762</v>
+        <v>313.8837336096964</v>
       </c>
       <c r="E65" t="n">
-        <v>316.7961120605469</v>
+        <v>316.796142578125</v>
       </c>
       <c r="F65" t="n">
         <v>31240900</v>
@@ -2136,16 +2136,16 @@
         <v>45996</v>
       </c>
       <c r="B66" t="n">
-        <v>318.6612638744486</v>
+        <v>318.6612335259534</v>
       </c>
       <c r="C66" t="n">
-        <v>322.3217576397153</v>
+        <v>322.3217269426038</v>
       </c>
       <c r="D66" t="n">
-        <v>318.3421170569229</v>
+        <v>318.3420867388224</v>
       </c>
       <c r="E66" t="n">
-        <v>320.4366455078125</v>
+        <v>320.4366149902344</v>
       </c>
       <c r="F66" t="n">
         <v>28851700</v>
@@ -2162,16 +2162,16 @@
         <v>45999</v>
       </c>
       <c r="B67" t="n">
-        <v>319.4285975207571</v>
+        <v>319.428628654094</v>
       </c>
       <c r="C67" t="n">
-        <v>319.8178549396436</v>
+        <v>319.8178861109197</v>
       </c>
       <c r="D67" t="n">
-        <v>310.6157547321785</v>
+        <v>310.6157850065654</v>
       </c>
       <c r="E67" t="n">
-        <v>313.1109008789062</v>
+        <v>313.1109313964844</v>
       </c>
       <c r="F67" t="n">
         <v>33909400</v>
@@ -2240,16 +2240,16 @@
         <v>46002</v>
       </c>
       <c r="B70" t="n">
-        <v>319.4585671045538</v>
+        <v>319.4585358397385</v>
       </c>
       <c r="C70" t="n">
-        <v>320.4965565243085</v>
+        <v>320.4965251579071</v>
       </c>
       <c r="D70" t="n">
-        <v>308.0008744502611</v>
+        <v>308.0008443067889</v>
       </c>
       <c r="E70" t="n">
-        <v>311.8234252929688</v>
+        <v>311.8233947753906</v>
       </c>
       <c r="F70" t="n">
         <v>42353700</v>
@@ -2292,16 +2292,16 @@
         <v>46006</v>
       </c>
       <c r="B72" t="n">
-        <v>310.7156001962807</v>
+        <v>310.7155693717638</v>
       </c>
       <c r="C72" t="n">
-        <v>310.8154121445851</v>
+        <v>310.8153813101663</v>
       </c>
       <c r="D72" t="n">
-        <v>304.2881005921093</v>
+        <v>304.288070405232</v>
       </c>
       <c r="E72" t="n">
-        <v>307.6216125488281</v>
+        <v>307.62158203125</v>
       </c>
       <c r="F72" t="n">
         <v>29151900</v>
@@ -2422,16 +2422,16 @@
         <v>46013</v>
       </c>
       <c r="B77" t="n">
-        <v>309.278400817878</v>
+        <v>309.2783702904479</v>
       </c>
       <c r="C77" t="n">
-        <v>309.5279154654388</v>
+        <v>309.5278849133803</v>
       </c>
       <c r="D77" t="n">
-        <v>304.707275417899</v>
+        <v>304.7072453416635</v>
       </c>
       <c r="E77" t="n">
-        <v>309.1785888671875</v>
+        <v>309.1785583496094</v>
       </c>
       <c r="F77" t="n">
         <v>26429900</v>
@@ -2474,16 +2474,16 @@
         <v>46015</v>
       </c>
       <c r="B79" t="n">
-        <v>314.1588359856885</v>
+        <v>314.1588665693361</v>
       </c>
       <c r="C79" t="n">
-        <v>314.4682316573388</v>
+        <v>314.4682622711062</v>
       </c>
       <c r="D79" t="n">
-        <v>311.3143938726672</v>
+        <v>311.3144241794057</v>
       </c>
       <c r="E79" t="n">
-        <v>313.4801635742188</v>
+        <v>313.4801940917969</v>
       </c>
       <c r="F79" t="n">
         <v>10097400</v>
@@ -2500,16 +2500,16 @@
         <v>46017</v>
       </c>
       <c r="B80" t="n">
-        <v>313.8694852656387</v>
+        <v>313.8694546536391</v>
       </c>
       <c r="C80" t="n">
-        <v>314.4782864028367</v>
+        <v>314.4782557314601</v>
       </c>
       <c r="D80" t="n">
-        <v>311.6737441219225</v>
+        <v>311.6737137240756</v>
       </c>
       <c r="E80" t="n">
-        <v>312.9013671875</v>
+        <v>312.9013366699219</v>
       </c>
       <c r="F80" t="n">
         <v>10899000</v>
@@ -2526,16 +2526,16 @@
         <v>46020</v>
       </c>
       <c r="B81" t="n">
-        <v>310.7655125785055</v>
+        <v>310.7654822740718</v>
       </c>
       <c r="C81" t="n">
-        <v>313.410361871903</v>
+        <v>313.4103313095557</v>
       </c>
       <c r="D81" t="n">
-        <v>310.0169686016006</v>
+        <v>310.0169383701615</v>
       </c>
       <c r="E81" t="n">
-        <v>312.9512634277344</v>
+        <v>312.9512329101562</v>
       </c>
       <c r="F81" t="n">
         <v>19621800</v>
@@ -2604,16 +2604,16 @@
         <v>46024</v>
       </c>
       <c r="B84" t="n">
-        <v>316.2847187538463</v>
+        <v>316.2847494408858</v>
       </c>
       <c r="C84" t="n">
-        <v>321.87385220157</v>
+        <v>321.8738834308866</v>
       </c>
       <c r="D84" t="n">
-        <v>309.7274673850438</v>
+        <v>309.727497435876</v>
       </c>
       <c r="E84" t="n">
-        <v>314.5381164550781</v>
+        <v>314.5381469726562</v>
       </c>
       <c r="F84" t="n">
         <v>32009400</v>
@@ -2630,16 +2630,16 @@
         <v>46027</v>
       </c>
       <c r="B85" t="n">
-        <v>317.0432662013207</v>
+        <v>317.0432968268774</v>
       </c>
       <c r="C85" t="n">
-        <v>318.4006111389099</v>
+        <v>318.4006418955826</v>
       </c>
       <c r="D85" t="n">
-        <v>314.0191501700305</v>
+        <v>314.0191805034655</v>
       </c>
       <c r="E85" t="n">
-        <v>315.9254455566406</v>
+        <v>315.9254760742188</v>
       </c>
       <c r="F85" t="n">
         <v>30195600</v>
@@ -2682,16 +2682,16 @@
         <v>46029</v>
       </c>
       <c r="B87" t="n">
-        <v>313.7496873061683</v>
+        <v>313.7496575108236</v>
       </c>
       <c r="C87" t="n">
-        <v>325.5168067446344</v>
+        <v>325.5167758318212</v>
       </c>
       <c r="D87" t="n">
-        <v>313.5800344006012</v>
+        <v>313.5800046213677</v>
       </c>
       <c r="E87" t="n">
-        <v>321.3549194335938</v>
+        <v>321.3548889160156</v>
       </c>
       <c r="F87" t="n">
         <v>35104400</v>
@@ -2760,16 +2760,16 @@
         <v>46034</v>
       </c>
       <c r="B90" t="n">
-        <v>325.1674658209474</v>
+        <v>325.1674358606418</v>
       </c>
       <c r="C90" t="n">
-        <v>333.3914890456728</v>
+        <v>333.3914583276215</v>
       </c>
       <c r="D90" t="n">
-        <v>324.3690311583512</v>
+        <v>324.3690012716118</v>
       </c>
       <c r="E90" t="n">
-        <v>331.2156982421875</v>
+        <v>331.2156677246094</v>
       </c>
       <c r="F90" t="n">
         <v>33923900</v>
@@ -2786,16 +2786,16 @@
         <v>46035</v>
       </c>
       <c r="B91" t="n">
-        <v>334.2996793666924</v>
+        <v>334.2997097916206</v>
       </c>
       <c r="C91" t="n">
-        <v>339.8289010736461</v>
+        <v>339.828932001794</v>
       </c>
       <c r="D91" t="n">
-        <v>332.9722446137951</v>
+        <v>332.9722749179122</v>
       </c>
       <c r="E91" t="n">
-        <v>335.3176879882812</v>
+        <v>335.3177185058594</v>
       </c>
       <c r="F91" t="n">
         <v>33517600</v>
@@ -2838,16 +2838,16 @@
         <v>46037</v>
       </c>
       <c r="B93" t="n">
-        <v>336.9944512235705</v>
+        <v>336.9944202593897</v>
       </c>
       <c r="C93" t="n">
-        <v>337.03438209247</v>
+        <v>337.0343511246202</v>
       </c>
       <c r="D93" t="n">
-        <v>330.097863235539</v>
+        <v>330.0978329050398</v>
       </c>
       <c r="E93" t="n">
-        <v>332.1339111328125</v>
+        <v>332.1338806152344</v>
       </c>
       <c r="F93" t="n">
         <v>28442400</v>
@@ -2942,16 +2942,16 @@
         <v>46044</v>
       </c>
       <c r="B97" t="n">
-        <v>333.8006666576773</v>
+        <v>333.8006975362521</v>
       </c>
       <c r="C97" t="n">
-        <v>334.4992893099707</v>
+        <v>334.4993202531722</v>
       </c>
       <c r="D97" t="n">
-        <v>328.1117212092731</v>
+        <v>328.1117515615861</v>
       </c>
       <c r="E97" t="n">
-        <v>329.8982543945312</v>
+        <v>329.8982849121094</v>
       </c>
       <c r="F97" t="n">
         <v>26253600</v>
@@ -3046,16 +3046,16 @@
         <v>46050</v>
       </c>
       <c r="B101" t="n">
-        <v>335.4075262381039</v>
+        <v>335.4075567602221</v>
       </c>
       <c r="C101" t="n">
-        <v>336.8846637353836</v>
+        <v>336.8846943919215</v>
       </c>
       <c r="D101" t="n">
-        <v>331.2955302242731</v>
+        <v>331.2955603721992</v>
       </c>
       <c r="E101" t="n">
-        <v>335.3576354980469</v>
+        <v>335.357666015625</v>
       </c>
       <c r="F101" t="n">
         <v>27434400</v>
@@ -3072,16 +3072,16 @@
         <v>46051</v>
       </c>
       <c r="B102" t="n">
-        <v>339.6393000059441</v>
+        <v>339.639269303412</v>
       </c>
       <c r="C102" t="n">
-        <v>341.625457159737</v>
+        <v>341.6254262776615</v>
       </c>
       <c r="D102" t="n">
-        <v>325.9060355700189</v>
+        <v>325.9060061089392</v>
       </c>
       <c r="E102" t="n">
-        <v>337.5932922363281</v>
+        <v>337.59326171875</v>
       </c>
       <c r="F102" t="n">
         <v>39785600</v>
@@ -3124,16 +3124,16 @@
         <v>46055</v>
       </c>
       <c r="B104" t="n">
-        <v>335.5672073695487</v>
+        <v>335.5672372238362</v>
       </c>
       <c r="C104" t="n">
-        <v>344.1604758527643</v>
+        <v>344.160506471566</v>
       </c>
       <c r="D104" t="n">
-        <v>334.9783565494149</v>
+        <v>334.9783863513143</v>
       </c>
       <c r="E104" t="n">
-        <v>343.022705078125</v>
+        <v>343.0227355957031</v>
       </c>
       <c r="F104" t="n">
         <v>32006100</v>
@@ -3176,16 +3176,16 @@
         <v>46057</v>
       </c>
       <c r="B106" t="n">
-        <v>342.2941565134455</v>
+        <v>342.2941250868659</v>
       </c>
       <c r="C106" t="n">
-        <v>342.6434831024425</v>
+        <v>342.6434516437907</v>
       </c>
       <c r="D106" t="n">
-        <v>327.8821884154679</v>
+        <v>327.8821583120744</v>
       </c>
       <c r="E106" t="n">
-        <v>332.3934326171875</v>
+        <v>332.3934020996094</v>
       </c>
       <c r="F106" t="n">
         <v>70618400</v>
@@ -3202,16 +3202,16 @@
         <v>46058</v>
       </c>
       <c r="B107" t="n">
-        <v>311.6138496060838</v>
+        <v>311.6138208417116</v>
       </c>
       <c r="C107" t="n">
-        <v>332.0441098613053</v>
+        <v>332.0440792110618</v>
       </c>
       <c r="D107" t="n">
-        <v>305.8650224655501</v>
+        <v>305.8649942318392</v>
       </c>
       <c r="E107" t="n">
-        <v>330.6069030761719</v>
+        <v>330.6068725585938</v>
       </c>
       <c r="F107" t="n">
         <v>88205800</v>
@@ -3306,16 +3306,16 @@
         <v>46064</v>
       </c>
       <c r="B111" t="n">
-        <v>318.3506892240785</v>
+        <v>318.3507205277581</v>
       </c>
       <c r="C111" t="n">
-        <v>320.4366276261131</v>
+        <v>320.4366591349046</v>
       </c>
       <c r="D111" t="n">
-        <v>309.0587679521403</v>
+        <v>309.0587983421378</v>
       </c>
       <c r="E111" t="n">
-        <v>310.3562316894531</v>
+        <v>310.3562622070312</v>
       </c>
       <c r="F111" t="n">
         <v>45406400</v>
@@ -3332,16 +3332,16 @@
         <v>46065</v>
       </c>
       <c r="B112" t="n">
-        <v>311.4840826487114</v>
+        <v>311.4840518259579</v>
       </c>
       <c r="C112" t="n">
-        <v>315.6260194522374</v>
+        <v>315.6259882196205</v>
       </c>
       <c r="D112" t="n">
-        <v>306.603592280419</v>
+        <v>306.603561940612</v>
       </c>
       <c r="E112" t="n">
-        <v>308.4000854492188</v>
+        <v>308.4000549316406</v>
       </c>
       <c r="F112" t="n">
         <v>47761300</v>
@@ -3462,16 +3462,16 @@
         <v>46073</v>
       </c>
       <c r="B117" t="n">
-        <v>303.7291917307074</v>
+        <v>303.7291622459488</v>
       </c>
       <c r="C117" t="n">
-        <v>315.8855378192499</v>
+        <v>315.885507154404</v>
       </c>
       <c r="D117" t="n">
-        <v>303.3099937290923</v>
+        <v>303.3099642850277</v>
       </c>
       <c r="E117" t="n">
-        <v>314.3684997558594</v>
+        <v>314.3684692382812</v>
       </c>
       <c r="F117" t="n">
         <v>53210800</v>
@@ -3540,16 +3540,16 @@
         <v>46078</v>
       </c>
       <c r="B120" t="n">
-        <v>311.4541454679639</v>
+        <v>311.4541150323118</v>
       </c>
       <c r="C120" t="n">
-        <v>313.031095017384</v>
+        <v>313.0310644276307</v>
       </c>
       <c r="D120" t="n">
-        <v>308.8392369672335</v>
+        <v>308.8392067871133</v>
       </c>
       <c r="E120" t="n">
-        <v>312.2925109863281</v>
+        <v>312.29248046875</v>
       </c>
       <c r="F120" t="n">
         <v>29963600</v>
@@ -3566,16 +3566,16 @@
         <v>46079</v>
       </c>
       <c r="B121" t="n">
-        <v>312.0330001798944</v>
+        <v>312.0330312197015</v>
       </c>
       <c r="C121" t="n">
-        <v>312.5320293917034</v>
+        <v>312.5320604811519</v>
       </c>
       <c r="D121" t="n">
-        <v>301.762970472535</v>
+        <v>301.7630004907203</v>
       </c>
       <c r="E121" t="n">
-        <v>306.783203125</v>
+        <v>306.7832336425781</v>
       </c>
       <c r="F121" t="n">
         <v>36431200</v>
@@ -3696,16 +3696,16 @@
         <v>46086</v>
       </c>
       <c r="B126" t="n">
-        <v>302.4516780897468</v>
+        <v>302.4516473530844</v>
       </c>
       <c r="C126" t="n">
-        <v>302.7111526067185</v>
+        <v>302.711121843687</v>
       </c>
       <c r="D126" t="n">
-        <v>297.4114640277728</v>
+        <v>297.4114338033223</v>
       </c>
       <c r="E126" t="n">
-        <v>300.2958679199219</v>
+        <v>300.2958374023438</v>
       </c>
       <c r="F126" t="n">
         <v>35752300</v>
@@ -10903,7 +10903,7 @@
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>2026-09-07 03:08:04</t>
+          <t>2026-09-08 08:51:55</t>
         </is>
       </c>
     </row>

</xml_diff>